<commit_message>
feat: análisis fila única, infogramas e insights abril 2026
- PDFs de análisis por hora/día (sábados, domingo, semana santa, fila única)
- Infogramas economía unitaria, cross-sell y roadmap 90 días
- Auditorías dataset y conclusiones BOSIN
- Corrección items marzo/abril 2026 + backup pre-fix
- Actualización scripts insight/costos y datasets

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nino/CrossSelling_NINO.xlsx
+++ b/nino/CrossSelling_NINO.xlsx
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Periodo: 16/02/2026 - 18/03/2026 (31 dias) | Que compran los clientes junto con Rotiseria?</t>
+          <t xml:space="preserve">  Periodo: 01/03/2026 - 31/03/2026 (31 dias) | Que compran los clientes junto con Rotiseria?</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>1159</v>
+        <v>1189</v>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr"/>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>11369307</v>
+        <v>10575200</v>
       </c>
       <c r="C7" s="7" t="inlineStr"/>
       <c r="D7" s="7" t="inlineStr"/>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>54272664</v>
+        <v>51580059</v>
       </c>
       <c r="C8" s="9" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>65641971</v>
+        <v>62155259</v>
       </c>
       <c r="C9" s="11" t="inlineStr"/>
       <c r="D9" s="11" t="inlineStr"/>
@@ -644,7 +644,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>4.8x</t>
+          <t>4.9x</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr"/>
@@ -653,7 +653,7 @@
       <c r="F10" s="13" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Por cada $1 de rotiseria, se venden $4.8 de otros rubros</t>
+          <t>Por cada $1 de rotiseria, se venden $4.9 de otros rubros</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>56637</v>
+        <v>52275</v>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr"/>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>31175</v>
+        <v>28718</v>
       </c>
       <c r="C13" s="7" t="inlineStr"/>
       <c r="D13" s="7" t="inlineStr"/>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>25462</v>
+        <v>23557</v>
       </c>
       <c r="C14" s="9" t="inlineStr"/>
       <c r="D14" s="9" t="inlineStr"/>
@@ -711,7 +711,7 @@
       <c r="F14" s="9" t="inlineStr"/>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>El cliente de rotiseria gasta $25,462 mas por ticket</t>
+          <t>El cliente de rotiseria gasta $23,557 mas por ticket</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>11155381</v>
+        <v>10376216</v>
       </c>
       <c r="C18" s="7" t="inlineStr"/>
       <c r="D18" s="7" t="inlineStr"/>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>53251462</v>
+        <v>50609522</v>
       </c>
       <c r="C19" s="9" t="inlineStr"/>
       <c r="D19" s="9" t="inlineStr"/>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>64406843</v>
+        <v>60985738</v>
       </c>
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr"/>
@@ -787,7 +787,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Si se cierra rotiseria, se perderian ~$53,251,462/mes en ventas de otros rubros (cross-sell)</t>
+          <t xml:space="preserve">  Si se cierra rotiseria, se perderian ~$50,609,522/mes en ventas de otros rubros (cross-sell)</t>
         </is>
       </c>
     </row>
@@ -842,24 +842,24 @@
         </is>
       </c>
       <c r="B25" s="15" t="n">
-        <v>12400657</v>
+        <v>12387053</v>
       </c>
       <c r="C25" s="15" t="n">
-        <v>820</v>
+        <v>774</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>357</v>
+        <v>387</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>30.8%</t>
+          <t>32.5%</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>34736</v>
+        <v>32008</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>12167325</v>
+        <v>12153976</v>
       </c>
     </row>
     <row r="26">
@@ -869,13 +869,13 @@
         </is>
       </c>
       <c r="B26" s="15" t="n">
-        <v>8404333</v>
+        <v>7624766</v>
       </c>
       <c r="C26" s="15" t="n">
-        <v>4224</v>
+        <v>3629</v>
       </c>
       <c r="D26" s="15" t="n">
-        <v>887</v>
+        <v>910</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -883,10 +883,10 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>9475</v>
+        <v>8379</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>8246196</v>
+        <v>7481298</v>
       </c>
     </row>
     <row r="27">
@@ -896,51 +896,51 @@
         </is>
       </c>
       <c r="B27" s="15" t="n">
-        <v>5495990</v>
+        <v>5216350</v>
       </c>
       <c r="C27" s="15" t="n">
-        <v>1553</v>
+        <v>1325</v>
       </c>
       <c r="D27" s="15" t="n">
-        <v>614</v>
+        <v>637</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>53.0%</t>
+          <t>53.6%</t>
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>8951</v>
+        <v>8189</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>5392577</v>
+        <v>5118199</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>BEBIDAS</t>
+          <t>FIAMBRERIA</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
-        <v>3634754</v>
+        <v>3358550</v>
       </c>
       <c r="C28" s="15" t="n">
-        <v>1219</v>
+        <v>856</v>
       </c>
       <c r="D28" s="15" t="n">
-        <v>529</v>
+        <v>478</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>45.6%</t>
+          <t>40.2%</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>6871</v>
+        <v>7026</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>3566362</v>
+        <v>3295355</v>
       </c>
     </row>
     <row r="29">
@@ -950,51 +950,51 @@
         </is>
       </c>
       <c r="B29" s="15" t="n">
-        <v>3321689</v>
+        <v>3223829</v>
       </c>
       <c r="C29" s="15" t="n">
-        <v>966</v>
+        <v>853</v>
       </c>
       <c r="D29" s="15" t="n">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>32.9%</t>
+          <t>31.6%</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>8718</v>
+        <v>8574</v>
       </c>
       <c r="G29" s="15" t="n">
-        <v>3259188</v>
+        <v>3163169</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>FIAMBRERIA</t>
+          <t>BEBIDAS</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
-        <v>3120905</v>
+        <v>3030711</v>
       </c>
       <c r="C30" s="15" t="n">
-        <v>835</v>
+        <v>910</v>
       </c>
       <c r="D30" s="15" t="n">
-        <v>460</v>
+        <v>501</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>6785</v>
+        <v>6049</v>
       </c>
       <c r="G30" s="15" t="n">
-        <v>3062182</v>
+        <v>2973685</v>
       </c>
     </row>
     <row r="31">
@@ -1004,24 +1004,24 @@
         </is>
       </c>
       <c r="B31" s="15" t="n">
-        <v>3091002</v>
+        <v>2867889</v>
       </c>
       <c r="C31" s="15" t="n">
-        <v>1143</v>
+        <v>1010</v>
       </c>
       <c r="D31" s="15" t="n">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>35.7%</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>7521</v>
+        <v>6748</v>
       </c>
       <c r="G31" s="15" t="n">
-        <v>3032841</v>
+        <v>2813926</v>
       </c>
     </row>
     <row r="32">
@@ -1031,240 +1031,240 @@
         </is>
       </c>
       <c r="B32" s="17" t="n">
-        <v>2393730</v>
+        <v>2238109</v>
       </c>
       <c r="C32" s="17" t="n">
-        <v>258</v>
+        <v>231</v>
       </c>
       <c r="D32" s="17" t="n">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="F32" s="17" t="n">
-        <v>12939</v>
+        <v>11419</v>
       </c>
       <c r="G32" s="17" t="n">
-        <v>2348689</v>
+        <v>2195997</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>ELABORADOS DE CARNICERIA</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>1356643</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>122</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>8.4%</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>13566</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>1331116</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>ART.DE 1RA NECESIDAD</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>1348132</v>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>410</v>
+      </c>
+      <c r="D34" s="17" t="n">
+        <v>288</v>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>24.2%</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="n">
+        <v>4681</v>
+      </c>
+      <c r="G34" s="17" t="n">
+        <v>1322765</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>PANAD.ELAB.PROPIA</t>
         </is>
       </c>
-      <c r="B33" s="15" t="n">
-        <v>1729924</v>
-      </c>
-      <c r="C33" s="15" t="n">
-        <v>1096</v>
-      </c>
-      <c r="D33" s="15" t="n">
-        <v>589</v>
-      </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>50.8%</t>
-        </is>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>2937</v>
-      </c>
-      <c r="G33" s="15" t="n">
-        <v>1697374</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>ELABORADOS DE CARNICERIA</t>
-        </is>
-      </c>
-      <c r="B34" s="8" t="n">
-        <v>1365387</v>
-      </c>
-      <c r="C34" s="8" t="n">
+      <c r="B35" s="15" t="n">
+        <v>1297189</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>561</v>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>47.2%</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>2312</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>1272781</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>REPOSTERIA Y PASTELERIA</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>1045771</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>158</v>
+      </c>
+      <c r="D36" s="8" t="n">
         <v>117</v>
       </c>
-      <c r="D34" s="18" t="n">
-        <v>92</v>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>7.9%</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="n">
-        <v>14841</v>
-      </c>
-      <c r="G34" s="8" t="n">
-        <v>1339696</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>ART.DE 1RA NECESIDAD</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="n">
-        <v>1330420</v>
-      </c>
-      <c r="C35" s="17" t="n">
-        <v>416</v>
-      </c>
-      <c r="D35" s="17" t="n">
-        <v>248</v>
-      </c>
-      <c r="E35" s="16" t="inlineStr">
-        <is>
-          <t>21.4%</t>
-        </is>
-      </c>
-      <c r="F35" s="17" t="n">
-        <v>5365</v>
-      </c>
-      <c r="G35" s="17" t="n">
-        <v>1305387</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>PANIFIC.Y MASAS FRESCAS</t>
-        </is>
-      </c>
-      <c r="B36" s="17" t="n">
-        <v>1175955</v>
-      </c>
-      <c r="C36" s="17" t="n">
-        <v>403</v>
-      </c>
-      <c r="D36" s="17" t="n">
-        <v>255</v>
-      </c>
-      <c r="E36" s="16" t="inlineStr">
-        <is>
-          <t>22.0%</t>
-        </is>
-      </c>
-      <c r="F36" s="17" t="n">
-        <v>4612</v>
-      </c>
-      <c r="G36" s="17" t="n">
-        <v>1153828</v>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>8938</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>1026093</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
         <is>
+          <t>PANIFIC.Y MASAS FRESCAS</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="n">
+        <v>1010150</v>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>335</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <v>270</v>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>22.7%</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="n">
+        <v>3741</v>
+      </c>
+      <c r="G37" s="17" t="n">
+        <v>991143</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
           <t>GOLOSINAS</t>
         </is>
       </c>
-      <c r="B37" s="17" t="n">
-        <v>1101392</v>
-      </c>
-      <c r="C37" s="17" t="n">
-        <v>503</v>
-      </c>
-      <c r="D37" s="17" t="n">
-        <v>256</v>
-      </c>
-      <c r="E37" s="16" t="inlineStr">
-        <is>
-          <t>22.1%</t>
-        </is>
-      </c>
-      <c r="F37" s="17" t="n">
-        <v>4302</v>
-      </c>
-      <c r="G37" s="17" t="n">
-        <v>1080668</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>REPOSTERIA Y PASTELERIA</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="n">
-        <v>1056281</v>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>161</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>117</v>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>10.1%</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="n">
-        <v>9028</v>
-      </c>
-      <c r="G38" s="8" t="n">
-        <v>1036406</v>
+      <c r="B38" s="17" t="n">
+        <v>973409</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>377</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <v>251</v>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>21.1%</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="n">
+        <v>3878</v>
+      </c>
+      <c r="G38" s="17" t="n">
+        <v>955093</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>EMBUTIDOS</t>
+          <t>BAZAR</t>
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>1042914</v>
+        <v>920116</v>
       </c>
       <c r="C39" s="8" t="n">
-        <v>167</v>
+        <v>214</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="F39" s="8" t="n">
-        <v>9069</v>
+        <v>6053</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>1023290</v>
+        <v>902803</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>BAZAR</t>
+          <t>EMBUTIDOS</t>
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>849456</v>
+        <v>906855</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>249</v>
+        <v>160</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>11.7%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="F40" s="8" t="n">
-        <v>6246</v>
+        <v>7621</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>833473</v>
+        <v>889791</v>
       </c>
     </row>
     <row r="41">
@@ -1274,24 +1274,24 @@
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>840100</v>
+        <v>702355</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>267</v>
+        <v>190</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="F41" s="8" t="n">
-        <v>5601</v>
+        <v>4417</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>824293</v>
+        <v>689139</v>
       </c>
     </row>
     <row r="42">
@@ -1301,51 +1301,51 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>497800</v>
+        <v>288290</v>
       </c>
       <c r="C42" s="18" t="n">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="D42" s="18" t="n">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>4.4%</t>
         </is>
       </c>
       <c r="F42" s="8" t="n">
-        <v>7778</v>
+        <v>5544</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>488433</v>
+        <v>282865</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>LIBRERIA</t>
+          <t>FACTURAS Y TORTITAS</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>177325</v>
-      </c>
-      <c r="C43" s="18" t="n">
-        <v>78</v>
-      </c>
-      <c r="D43" s="18" t="n">
-        <v>40</v>
+        <v>247250</v>
+      </c>
+      <c r="C43" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>107</v>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>9.0%</t>
         </is>
       </c>
       <c r="F43" s="8" t="n">
-        <v>4433</v>
+        <v>2311</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>173988</v>
+        <v>242598</v>
       </c>
     </row>
     <row r="44">
@@ -1355,105 +1355,105 @@
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>173920</v>
+        <v>232590</v>
       </c>
       <c r="C44" s="18" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D44" s="18" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>1.3%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="F44" s="8" t="n">
-        <v>11595</v>
+        <v>9691</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>170647</v>
+        <v>228214</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>PESCADOS Y MARISCOS CONGELADOS</t>
+          <t>COTILLON</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>166835</v>
+        <v>199450</v>
       </c>
       <c r="C45" s="18" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="D45" s="18" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>1.1%</t>
+          <t>3.1%</t>
         </is>
       </c>
       <c r="F45" s="8" t="n">
-        <v>12833</v>
+        <v>5391</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>163696</v>
+        <v>195697</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>HUEVOS FRESCOS</t>
+          <t>PASCUA</t>
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>159550</v>
+        <v>198290</v>
       </c>
       <c r="C46" s="18" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="D46" s="18" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="F46" s="8" t="n">
-        <v>2346</v>
+        <v>9013</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>156548</v>
+        <v>194559</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>COTILLON</t>
+          <t>PESCADOS Y MARISCOS CONGELADOS</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>155942</v>
+        <v>181130</v>
       </c>
       <c r="C47" s="18" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D47" s="18" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="F47" s="8" t="n">
-        <v>4587</v>
+        <v>10063</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>153008</v>
+        <v>177721</v>
       </c>
     </row>
     <row r="48">
@@ -1463,304 +1463,304 @@
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>117400</v>
+        <v>137700</v>
       </c>
       <c r="C48" s="18" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D48" s="18" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="F48" s="8" t="n">
-        <v>5104</v>
+        <v>4590</v>
       </c>
       <c r="G48" s="8" t="n">
-        <v>115191</v>
+        <v>135109</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>HARINAS</t>
+          <t>LIBRERIA</t>
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>102835</v>
+        <v>116710</v>
       </c>
       <c r="C49" s="18" t="n">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>4.2%</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="F49" s="8" t="n">
-        <v>2099</v>
+        <v>3335</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>100900</v>
+        <v>114514</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>PASCUA</t>
+          <t>HARINAS</t>
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>98960</v>
+        <v>109155</v>
       </c>
       <c r="C50" s="18" t="n">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="D50" s="18" t="n">
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>0.6%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="F50" s="8" t="n">
-        <v>14137</v>
+        <v>1949</v>
       </c>
       <c r="G50" s="8" t="n">
-        <v>97098</v>
+        <v>107101</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>LEGUMBRES Y CEREALES 10,5% IVA</t>
+          <t>ENVASES VENTA</t>
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>76905</v>
+        <v>92330</v>
       </c>
       <c r="C51" s="18" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D51" s="18" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="F51" s="8" t="n">
-        <v>2262</v>
+        <v>2198</v>
       </c>
       <c r="G51" s="8" t="n">
-        <v>75458</v>
+        <v>90593</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>FERRETERIA</t>
+          <t>HUEVOS FRESCOS</t>
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>67160</v>
+        <v>86950</v>
       </c>
       <c r="C52" s="18" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>0.9%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="F52" s="8" t="n">
-        <v>6716</v>
+        <v>2229</v>
       </c>
       <c r="G52" s="8" t="n">
-        <v>65896</v>
+        <v>85314</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>ZAPATERIA</t>
+          <t>LEGUMBRES Y CEREALES 10,5% IVA</t>
         </is>
       </c>
       <c r="B53" s="8" t="n">
-        <v>25600</v>
+        <v>72820</v>
       </c>
       <c r="C53" s="18" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="D53" s="18" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="F53" s="8" t="n">
-        <v>12800</v>
+        <v>1867</v>
       </c>
       <c r="G53" s="8" t="n">
-        <v>25118</v>
+        <v>71450</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>LIBROS DE TEXTOS</t>
+          <t>FERRETERIA</t>
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>23600</v>
+        <v>50975</v>
       </c>
       <c r="C54" s="18" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D54" s="18" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>1.3%</t>
         </is>
       </c>
       <c r="F54" s="8" t="n">
-        <v>5900</v>
+        <v>3398</v>
       </c>
       <c r="G54" s="8" t="n">
-        <v>23156</v>
+        <v>50016</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>FACTURAS Y TORTITAS</t>
+          <t>JUGUETERIA</t>
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>17450</v>
+        <v>23625</v>
       </c>
       <c r="C55" s="18" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D55" s="18" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>0.8%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="F55" s="8" t="n">
-        <v>1939</v>
+        <v>23625</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>17122</v>
+        <v>23180</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>PRODUCTOS NAVIDEÑOS</t>
+          <t>CONGELADOS AL 10.5%</t>
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>8700</v>
+        <v>18676</v>
       </c>
       <c r="C56" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D56" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>0.5%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="F56" s="8" t="n">
-        <v>1450</v>
+        <v>3735</v>
       </c>
       <c r="G56" s="8" t="n">
-        <v>8536</v>
+        <v>18325</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>CONGELADOS AL 10.5%</t>
+          <t>PRODUCTOS NAVIDEÑOS</t>
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>8300</v>
+        <v>5460</v>
       </c>
       <c r="C57" s="18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D57" s="18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>0.3%</t>
         </is>
       </c>
       <c r="F57" s="8" t="n">
-        <v>8300</v>
+        <v>1365</v>
       </c>
       <c r="G57" s="8" t="n">
-        <v>8144</v>
+        <v>5357</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>PRODUCTOS PARA CARNEO</t>
+          <t>LIBROS DE TEXTOS</t>
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>6600</v>
+        <v>5200</v>
       </c>
       <c r="C58" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="F58" s="8" t="n">
-        <v>6600</v>
+        <v>2600</v>
       </c>
       <c r="G58" s="8" t="n">
-        <v>6476</v>
+        <v>5102</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>MEDICAMENTOS</t>
+          <t>IVA RED IB GRAL</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>1380</v>
+        <v>1850</v>
       </c>
       <c r="C59" s="18" t="n">
         <v>1</v>
@@ -1774,37 +1774,37 @@
         </is>
       </c>
       <c r="F59" s="8" t="n">
-        <v>1380</v>
+        <v>1850</v>
       </c>
       <c r="G59" s="8" t="n">
-        <v>1354</v>
+        <v>1815</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>ENVASES VENTA</t>
-        </is>
-      </c>
-      <c r="B60" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C60" s="8" t="n">
-        <v>128</v>
+          <t>MEDICAMENTOS</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="n">
+        <v>1380</v>
+      </c>
+      <c r="C60" s="18" t="n">
+        <v>1</v>
       </c>
       <c r="D60" s="18" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>4.3%</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="18" t="n">
-        <v>0</v>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G60" s="8" t="n">
+        <v>1354</v>
       </c>
     </row>
     <row r="61">
@@ -1814,16 +1814,16 @@
         </is>
       </c>
       <c r="B61" s="12" t="n">
-        <v>54272664</v>
+        <v>51580059</v>
       </c>
       <c r="C61" s="12" t="n">
-        <v>15073</v>
+        <v>12945</v>
       </c>
       <c r="D61" s="11" t="inlineStr"/>
       <c r="E61" s="11" t="inlineStr"/>
       <c r="F61" s="11" t="inlineStr"/>
       <c r="G61" s="12" t="n">
-        <v>53251462</v>
+        <v>50609522</v>
       </c>
     </row>
     <row r="62">
@@ -1885,41 +1885,41 @@
         </is>
       </c>
       <c r="C66" s="8" t="n">
-        <v>1443840</v>
+        <v>1468519</v>
       </c>
       <c r="D66" s="18" t="n">
         <v>88</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F66" s="8" t="n">
-        <v>14438</v>
+        <v>13350</v>
       </c>
       <c r="G66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>POLLO</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>MUSLO DE POLLO</t>
+          <t>COSTILLA ARQUEADA</t>
         </is>
       </c>
       <c r="C67" s="8" t="n">
-        <v>1001996</v>
-      </c>
-      <c r="D67" s="8" t="n">
-        <v>127</v>
-      </c>
-      <c r="E67" s="8" t="n">
-        <v>100</v>
+        <v>1022107</v>
+      </c>
+      <c r="D67" s="18" t="n">
+        <v>56</v>
+      </c>
+      <c r="E67" s="18" t="n">
+        <v>34</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>10020</v>
+        <v>30062</v>
       </c>
       <c r="G67" s="7" t="inlineStr"/>
     </row>
@@ -1931,45 +1931,45 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>COSTILLA ARQUEADA</t>
+          <t>FILET / LOMO</t>
         </is>
       </c>
       <c r="C68" s="8" t="n">
-        <v>954568</v>
+        <v>974006</v>
       </c>
       <c r="D68" s="18" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="E68" s="18" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>28926</v>
+        <v>22136</v>
       </c>
       <c r="G68" s="7" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>POLLO</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>FILET / LOMO</t>
+          <t>MUSLO DE POLLO</t>
         </is>
       </c>
       <c r="C69" s="8" t="n">
-        <v>948259</v>
-      </c>
-      <c r="D69" s="18" t="n">
-        <v>38</v>
-      </c>
-      <c r="E69" s="18" t="n">
-        <v>36</v>
+        <v>916321</v>
+      </c>
+      <c r="D69" s="8" t="n">
+        <v>116</v>
+      </c>
+      <c r="E69" s="8" t="n">
+        <v>100</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>26341</v>
+        <v>9163</v>
       </c>
       <c r="G69" s="7" t="inlineStr"/>
     </row>
@@ -1985,16 +1985,16 @@
         </is>
       </c>
       <c r="C70" s="8" t="n">
-        <v>838306</v>
+        <v>804850</v>
       </c>
       <c r="D70" s="18" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E70" s="18" t="n">
         <v>62</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>13521</v>
+        <v>12981</v>
       </c>
       <c r="G70" s="7" t="inlineStr"/>
     </row>
@@ -2006,20 +2006,20 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>MOLIDA INTERMEDIA</t>
+          <t>COSTELETA</t>
         </is>
       </c>
       <c r="C71" s="8" t="n">
-        <v>768650</v>
+        <v>702150</v>
       </c>
       <c r="D71" s="18" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="E71" s="18" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>15373</v>
+        <v>18004</v>
       </c>
       <c r="G71" s="7" t="inlineStr"/>
     </row>
@@ -2031,45 +2031,45 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>MILANESAS DE CARNE NINO</t>
+          <t>MILANESAS DE POLLO NINO</t>
         </is>
       </c>
       <c r="C72" s="8" t="n">
-        <v>695898</v>
+        <v>652520</v>
       </c>
       <c r="D72" s="18" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E72" s="18" t="n">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>15816</v>
+        <v>11060</v>
       </c>
       <c r="G72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>ELABORADOS DE CARNICERIA</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>PUNTA DE ESPALDA</t>
+          <t>MILANESAS DE CARNE NINO</t>
         </is>
       </c>
       <c r="C73" s="8" t="n">
-        <v>592030</v>
+        <v>610428</v>
       </c>
       <c r="D73" s="18" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E73" s="18" t="n">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>34825</v>
+        <v>14196</v>
       </c>
       <c r="G73" s="7" t="inlineStr"/>
     </row>
@@ -2081,20 +2081,20 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>COSTELETA</t>
+          <t>MOLIDA INTERMEDIA</t>
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>584526</v>
+        <v>567525</v>
       </c>
       <c r="D74" s="18" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E74" s="18" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="F74" s="8" t="n">
-        <v>18856</v>
+        <v>12338</v>
       </c>
       <c r="G74" s="7" t="inlineStr"/>
     </row>
@@ -2106,45 +2106,45 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>CUADRIL</t>
+          <t>VACIO</t>
         </is>
       </c>
       <c r="C75" s="8" t="n">
-        <v>583496</v>
+        <v>512828</v>
       </c>
       <c r="D75" s="18" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>17162</v>
+        <v>42736</v>
       </c>
       <c r="G75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>ELABORADOS DE CARNICERIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>MILANESAS DE POLLO NINO</t>
+          <t>CUADRIL</t>
         </is>
       </c>
       <c r="C76" s="8" t="n">
-        <v>580525</v>
+        <v>478152</v>
       </c>
       <c r="D76" s="18" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="E76" s="18" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>11610</v>
+        <v>19126</v>
       </c>
       <c r="G76" s="7" t="inlineStr"/>
     </row>
@@ -2156,20 +2156,20 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>NALGA</t>
+          <t>PUNTA DE ESPALDA</t>
         </is>
       </c>
       <c r="C77" s="8" t="n">
-        <v>498492</v>
+        <v>457840</v>
       </c>
       <c r="D77" s="18" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E77" s="18" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>20770</v>
+        <v>38153</v>
       </c>
       <c r="G77" s="7" t="inlineStr"/>
     </row>
@@ -2181,70 +2181,70 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>BOLA LOMO</t>
+          <t>NALGA</t>
         </is>
       </c>
       <c r="C78" s="8" t="n">
-        <v>478530</v>
+        <v>441296</v>
       </c>
       <c r="D78" s="18" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E78" s="18" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F78" s="8" t="n">
-        <v>17090</v>
+        <v>19187</v>
       </c>
       <c r="G78" s="7" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>EMBUTIDOS</t>
+          <t>FIAMBRERIA</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>CHORIZO PURO CERDO</t>
+          <t>PALADINI JAMON COCIDO</t>
         </is>
       </c>
       <c r="C79" s="8" t="n">
-        <v>440220</v>
+        <v>407945</v>
       </c>
       <c r="D79" s="18" t="n">
-        <v>33</v>
-      </c>
-      <c r="E79" s="18" t="n">
-        <v>48</v>
+        <v>24</v>
+      </c>
+      <c r="E79" s="8" t="n">
+        <v>100</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>9171</v>
+        <v>4079</v>
       </c>
       <c r="G79" s="7" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>POLLO</t>
+          <t>EMBUTIDOS</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>POLLO AVICOLA LUJAN</t>
+          <t>CHORIZO PURO CERDO</t>
         </is>
       </c>
       <c r="C80" s="8" t="n">
-        <v>415436</v>
+        <v>394442</v>
       </c>
       <c r="D80" s="18" t="n">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="E80" s="18" t="n">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="F80" s="8" t="n">
-        <v>15387</v>
+        <v>7044</v>
       </c>
       <c r="G80" s="7" t="inlineStr"/>
     </row>
@@ -2256,20 +2256,20 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>VACIO</t>
+          <t>BOLA LOMO</t>
         </is>
       </c>
       <c r="C81" s="8" t="n">
-        <v>379214</v>
+        <v>359945</v>
       </c>
       <c r="D81" s="18" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E81" s="18" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>34474</v>
+        <v>17997</v>
       </c>
       <c r="G81" s="7" t="inlineStr"/>
     </row>
@@ -2285,91 +2285,91 @@
         </is>
       </c>
       <c r="C82" s="8" t="n">
-        <v>377099</v>
+        <v>354060</v>
       </c>
       <c r="D82" s="18" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E82" s="18" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F82" s="8" t="n">
-        <v>25140</v>
+        <v>29505</v>
       </c>
       <c r="G82" s="7" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t>PANAD.ELAB.PROPIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>TORTAS NINO X 6U.</t>
+          <t>CUADRADA</t>
         </is>
       </c>
       <c r="C83" s="8" t="n">
-        <v>330400</v>
-      </c>
-      <c r="D83" s="8" t="n">
-        <v>200</v>
-      </c>
-      <c r="E83" s="8" t="n">
-        <v>153</v>
+        <v>349234</v>
+      </c>
+      <c r="D83" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="E83" s="18" t="n">
+        <v>18</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>2159</v>
+        <v>19402</v>
       </c>
       <c r="G83" s="7" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>ART.DE 1RA NECESIDAD</t>
+          <t>POLLO</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>HUEVOS FRESCOS MEDIO MAPLE</t>
+          <t>POLLO AVICOLA LUJAN</t>
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>328400</v>
+        <v>334264</v>
       </c>
       <c r="D84" s="18" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E84" s="18" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="F84" s="8" t="n">
-        <v>4499</v>
+        <v>12856</v>
       </c>
       <c r="G84" s="7" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>FIAMBRERIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>PALADINI JAMON COCIDO</t>
+          <t>COSTELETA BAJA</t>
         </is>
       </c>
       <c r="C85" s="8" t="n">
-        <v>319334</v>
+        <v>313614</v>
       </c>
       <c r="D85" s="18" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E85" s="18" t="n">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>3992</v>
+        <v>14934</v>
       </c>
       <c r="G85" s="7" t="inlineStr"/>
     </row>
@@ -2381,95 +2381,95 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>ILOLAY QUESO BARRRA</t>
+          <t>CREMOSO PUNTA DE AGUA</t>
         </is>
       </c>
       <c r="C86" s="8" t="n">
-        <v>286223</v>
+        <v>300802</v>
       </c>
       <c r="D86" s="18" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E86" s="18" t="n">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="F86" s="8" t="n">
-        <v>3180</v>
+        <v>5676</v>
       </c>
       <c r="G86" s="7" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>LACTEOS</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>CUADRADA</t>
+          <t>ILOLAY QUESO BARRRA</t>
         </is>
       </c>
       <c r="C87" s="8" t="n">
-        <v>280202</v>
+        <v>297167</v>
       </c>
       <c r="D87" s="18" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E87" s="18" t="n">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>17513</v>
+        <v>3266</v>
       </c>
       <c r="G87" s="7" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>EMBUTIDOS</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>MORCILLA VALENCIANA</t>
+          <t>PECETO</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>253267</v>
+        <v>285690</v>
       </c>
       <c r="D88" s="18" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E88" s="18" t="n">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="F88" s="8" t="n">
-        <v>5169</v>
+        <v>17856</v>
       </c>
       <c r="G88" s="7" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>ART.DE 1RA NECESIDAD</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>COSTILLA DE CERDO</t>
+          <t>HUEVOS FRESCOS MEDIO MAPLE</t>
         </is>
       </c>
       <c r="C89" s="8" t="n">
-        <v>251254</v>
+        <v>284900</v>
       </c>
       <c r="D89" s="18" t="n">
-        <v>31</v>
+        <v>77</v>
       </c>
       <c r="E89" s="18" t="n">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>9664</v>
+        <v>3799</v>
       </c>
       <c r="G89" s="7" t="inlineStr"/>
     </row>
@@ -2481,45 +2481,45 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>COSTELETA BAJA</t>
+          <t>PUNTA DE PIERNA</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>241714</v>
+        <v>282107</v>
       </c>
       <c r="D90" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E90" s="18" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F90" s="8" t="n">
-        <v>13429</v>
+        <v>18807</v>
       </c>
       <c r="G90" s="7" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>PANAD.ELAB.PROPIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>PAN NINO FLAUTA</t>
+          <t>COSTILLA DE CERDO</t>
         </is>
       </c>
       <c r="C91" s="8" t="n">
-        <v>241175</v>
-      </c>
-      <c r="D91" s="8" t="n">
-        <v>110</v>
-      </c>
-      <c r="E91" s="8" t="n">
-        <v>158</v>
+        <v>239376</v>
+      </c>
+      <c r="D91" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="E91" s="18" t="n">
+        <v>25</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>1526</v>
+        <v>9575</v>
       </c>
       <c r="G91" s="7" t="inlineStr"/>
     </row>
@@ -2531,70 +2531,70 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>PECETO</t>
+          <t>TAPA DE NALGA</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>238119</v>
+        <v>235313</v>
       </c>
       <c r="D92" s="18" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E92" s="18" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F92" s="8" t="n">
-        <v>19843</v>
+        <v>23531</v>
       </c>
       <c r="G92" s="7" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>BEBIDAS</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>FERNET BRANCA x 750 CC</t>
+          <t>ASADO RUSO</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>234300</v>
+        <v>231214</v>
       </c>
       <c r="D93" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="E93" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="E93" s="18" t="n">
-        <v>14</v>
-      </c>
       <c r="F93" s="8" t="n">
-        <v>16736</v>
+        <v>15414</v>
       </c>
       <c r="G93" s="7" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>LACTEOS</t>
+          <t>PANAD.ELAB.PROPIA</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>BARRA SANTA MARIA</t>
+          <t>PAN NINO FLAUTA</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>233066</v>
-      </c>
-      <c r="D94" s="18" t="n">
-        <v>21</v>
-      </c>
-      <c r="E94" s="18" t="n">
-        <v>82</v>
+        <v>230428</v>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E94" s="8" t="n">
+        <v>157</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>2842</v>
+        <v>1468</v>
       </c>
       <c r="G94" s="7" t="inlineStr"/>
     </row>
@@ -2610,16 +2610,16 @@
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>228656</v>
+        <v>226058</v>
       </c>
       <c r="D95" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="E95" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="E95" s="18" t="n">
-        <v>11</v>
-      </c>
       <c r="F95" s="8" t="n">
-        <v>20787</v>
+        <v>22606</v>
       </c>
       <c r="G95" s="7" t="inlineStr"/>
     </row>
@@ -2666,7 +2666,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Periodo: 16/02/2026 - 18/03/2026 (31 dias) | Que compran los clientes junto con Panaderia?</t>
+          <t xml:space="preserve">  Periodo: 01/03/2026 - 31/03/2026 (31 dias) | Que compran los clientes junto con Panaderia?</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>9983</v>
+        <v>9334</v>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr"/>
@@ -2716,7 +2716,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>28222420</v>
+        <v>20896544</v>
       </c>
       <c r="C7" s="7" t="inlineStr"/>
       <c r="D7" s="7" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>355826231</v>
+        <v>318496625</v>
       </c>
       <c r="C8" s="9" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>384048650</v>
+        <v>339393168</v>
       </c>
       <c r="C9" s="11" t="inlineStr"/>
       <c r="D9" s="11" t="inlineStr"/>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>12.6x</t>
+          <t>15.2x</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr"/>
@@ -2771,7 +2771,7 @@
       <c r="F10" s="13" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Por cada $1 de panaderia, se venden $12.6 de otros rubros</t>
+          <t>Por cada $1 de panaderia, se venden $15.2 de otros rubros</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>38470</v>
+        <v>36361</v>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr"/>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>28286</v>
+        <v>25978</v>
       </c>
       <c r="C13" s="7" t="inlineStr"/>
       <c r="D13" s="7" t="inlineStr"/>
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>10185</v>
+        <v>10383</v>
       </c>
       <c r="C14" s="9" t="inlineStr"/>
       <c r="D14" s="9" t="inlineStr"/>
@@ -2829,7 +2829,7 @@
       <c r="F14" s="9" t="inlineStr"/>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>El cliente de panaderia gasta $10,185 mas por ticket</t>
+          <t>El cliente de panaderia gasta $10,383 mas por ticket</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>27691383</v>
+        <v>20503352</v>
       </c>
       <c r="C18" s="7" t="inlineStr"/>
       <c r="D18" s="7" t="inlineStr"/>
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>349130958</v>
+        <v>312503751</v>
       </c>
       <c r="C19" s="9" t="inlineStr"/>
       <c r="D19" s="9" t="inlineStr"/>
@@ -2894,7 +2894,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>376822341</v>
+        <v>333007103</v>
       </c>
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr"/>
@@ -2905,7 +2905,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Si se cierra panaderia, se perderian ~$349,130,958/mes en ventas de otros rubros (cross-sell)</t>
+          <t xml:space="preserve">  Si se cierra panaderia, se perderian ~$312,503,751/mes en ventas de otros rubros (cross-sell)</t>
         </is>
       </c>
     </row>
@@ -2960,24 +2960,24 @@
         </is>
       </c>
       <c r="B25" s="15" t="n">
-        <v>94021669</v>
+        <v>88364695</v>
       </c>
       <c r="C25" s="15" t="n">
-        <v>6712</v>
+        <v>6038</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>3373</v>
+        <v>3206</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>33.8%</t>
+          <t>34.3%</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>27875</v>
+        <v>27562</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>92252545</v>
+        <v>86702014</v>
       </c>
     </row>
     <row r="26">
@@ -2987,24 +2987,24 @@
         </is>
       </c>
       <c r="B26" s="15" t="n">
-        <v>57957640</v>
+        <v>48534140</v>
       </c>
       <c r="C26" s="15" t="n">
-        <v>33007</v>
+        <v>25602</v>
       </c>
       <c r="D26" s="15" t="n">
-        <v>7458</v>
+        <v>6990</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>74.7%</t>
+          <t>74.9%</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>7771</v>
+        <v>6943</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>56867102</v>
+        <v>47620915</v>
       </c>
     </row>
     <row r="27">
@@ -3014,159 +3014,159 @@
         </is>
       </c>
       <c r="B27" s="15" t="n">
-        <v>33172565</v>
+        <v>29150403</v>
       </c>
       <c r="C27" s="15" t="n">
-        <v>10152</v>
+        <v>7991</v>
       </c>
       <c r="D27" s="15" t="n">
-        <v>4697</v>
+        <v>4477</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>7063</v>
+        <v>6511</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>32548386</v>
+        <v>28601906</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>PERFUMERIA</t>
+          <t>POLLO</t>
         </is>
       </c>
       <c r="B28" s="17" t="n">
-        <v>21747264</v>
+        <v>19644752</v>
       </c>
       <c r="C28" s="17" t="n">
-        <v>6986</v>
+        <v>2015</v>
       </c>
       <c r="D28" s="17" t="n">
-        <v>2892</v>
+        <v>1684</v>
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="F28" s="17" t="n">
-        <v>7520</v>
+        <v>11666</v>
       </c>
       <c r="G28" s="17" t="n">
-        <v>21338065</v>
+        <v>19275114</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>POLLO</t>
+          <t>PERFUMERIA</t>
         </is>
       </c>
       <c r="B29" s="17" t="n">
-        <v>20669953</v>
+        <v>18384883</v>
       </c>
       <c r="C29" s="17" t="n">
-        <v>2322</v>
+        <v>5558</v>
       </c>
       <c r="D29" s="17" t="n">
-        <v>1738</v>
+        <v>2711</v>
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>29.0%</t>
         </is>
       </c>
       <c r="F29" s="17" t="n">
-        <v>11893</v>
+        <v>6782</v>
       </c>
       <c r="G29" s="17" t="n">
-        <v>20281024</v>
+        <v>18038951</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>LIMPIEZA</t>
+          <t>FIAMBRERIA</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
-        <v>19815477</v>
+        <v>18129906</v>
       </c>
       <c r="C30" s="15" t="n">
-        <v>8074</v>
+        <v>5668</v>
       </c>
       <c r="D30" s="15" t="n">
-        <v>3329</v>
+        <v>3439</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>36.8%</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>5952</v>
+        <v>5272</v>
       </c>
       <c r="G30" s="15" t="n">
-        <v>19442626</v>
+        <v>17788771</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>BEBIDAS</t>
+          <t>LIMPIEZA</t>
         </is>
       </c>
       <c r="B31" s="15" t="n">
-        <v>18634578</v>
+        <v>17326605</v>
       </c>
       <c r="C31" s="15" t="n">
-        <v>7594</v>
+        <v>6619</v>
       </c>
       <c r="D31" s="15" t="n">
-        <v>3597</v>
+        <v>3076</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>33.0%</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>5181</v>
+        <v>5633</v>
       </c>
       <c r="G31" s="15" t="n">
-        <v>18283947</v>
+        <v>17000585</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>FIAMBRERIA</t>
+          <t>BEBIDAS</t>
         </is>
       </c>
       <c r="B32" s="15" t="n">
-        <v>18584141</v>
+        <v>15059559</v>
       </c>
       <c r="C32" s="15" t="n">
-        <v>6358</v>
+        <v>5264</v>
       </c>
       <c r="D32" s="15" t="n">
-        <v>3498</v>
+        <v>3282</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>35.0%</t>
+          <t>35.2%</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>5313</v>
+        <v>4589</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>18234459</v>
+        <v>14776196</v>
       </c>
     </row>
     <row r="33">
@@ -3176,24 +3176,24 @@
         </is>
       </c>
       <c r="B33" s="17" t="n">
-        <v>11036995</v>
+        <v>10171202</v>
       </c>
       <c r="C33" s="17" t="n">
-        <v>3742</v>
+        <v>3334</v>
       </c>
       <c r="D33" s="17" t="n">
-        <v>2295</v>
+        <v>2374</v>
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="F33" s="17" t="n">
-        <v>4809</v>
+        <v>4284</v>
       </c>
       <c r="G33" s="17" t="n">
-        <v>10829321</v>
+        <v>9979819</v>
       </c>
     </row>
     <row r="34">
@@ -3203,24 +3203,24 @@
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>9292810</v>
+        <v>8499784</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>816</v>
+        <v>780</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.3%</t>
         </is>
       </c>
       <c r="F34" s="8" t="n">
-        <v>13468</v>
+        <v>12463</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>9117955</v>
+        <v>8339851</v>
       </c>
     </row>
     <row r="35">
@@ -3230,24 +3230,24 @@
         </is>
       </c>
       <c r="B35" s="17" t="n">
-        <v>7222410</v>
+        <v>5899000</v>
       </c>
       <c r="C35" s="17" t="n">
-        <v>2845</v>
+        <v>2140</v>
       </c>
       <c r="D35" s="17" t="n">
-        <v>1767</v>
+        <v>1694</v>
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="F35" s="17" t="n">
-        <v>4087</v>
+        <v>3482</v>
       </c>
       <c r="G35" s="17" t="n">
-        <v>7086512</v>
+        <v>5788004</v>
       </c>
     </row>
     <row r="36">
@@ -3257,78 +3257,78 @@
         </is>
       </c>
       <c r="B36" s="17" t="n">
-        <v>5974541</v>
+        <v>5381311</v>
       </c>
       <c r="C36" s="17" t="n">
-        <v>3294</v>
+        <v>2496</v>
       </c>
       <c r="D36" s="17" t="n">
-        <v>1842</v>
+        <v>1750</v>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="F36" s="17" t="n">
-        <v>3244</v>
+        <v>3075</v>
       </c>
       <c r="G36" s="17" t="n">
-        <v>5862124</v>
+        <v>5280056</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>ROTISERIA</t>
+          <t>EMBUTIDOS</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>5594672</v>
+        <v>4852392</v>
       </c>
       <c r="C37" s="8" t="n">
-        <v>947</v>
+        <v>844</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>589</v>
+        <v>647</v>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="F37" s="8" t="n">
-        <v>9499</v>
+        <v>7500</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>5489402</v>
+        <v>4761089</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>EMBUTIDOS</t>
+          <t>ROTISERIA</t>
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>5453682</v>
+        <v>4817212</v>
       </c>
       <c r="C38" s="8" t="n">
-        <v>965</v>
+        <v>763</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>663</v>
+        <v>561</v>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="F38" s="8" t="n">
-        <v>8226</v>
+        <v>8587</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>5351065</v>
+        <v>4726571</v>
       </c>
     </row>
     <row r="39">
@@ -3338,24 +3338,24 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>5422124</v>
+        <v>4713936</v>
       </c>
       <c r="C39" s="8" t="n">
-        <v>1634</v>
+        <v>1155</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>970</v>
+        <v>883</v>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="F39" s="8" t="n">
-        <v>5590</v>
+        <v>5339</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>5320100</v>
+        <v>4625238</v>
       </c>
     </row>
     <row r="40">
@@ -3365,24 +3365,24 @@
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>5171285</v>
+        <v>3551300</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>2227</v>
+        <v>1370</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>1278</v>
+        <v>1229</v>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="F40" s="8" t="n">
-        <v>4046</v>
+        <v>2890</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>5073981</v>
+        <v>3484478</v>
       </c>
     </row>
     <row r="41">
@@ -3392,67 +3392,67 @@
         </is>
       </c>
       <c r="B41" s="8" t="n">
-        <v>3576502</v>
+        <v>3454761</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>480</v>
+        <v>464</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>3.9%</t>
+          <t>4.1%</t>
         </is>
       </c>
       <c r="F41" s="8" t="n">
-        <v>9171</v>
+        <v>9044</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>3509206</v>
+        <v>3389756</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>CONGELADOS HELADOS</t>
+          <t>FACTURAS Y TORTITAS</t>
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>2629265</v>
+        <v>2427150</v>
       </c>
       <c r="C42" s="8" t="n">
-        <v>640</v>
+        <v>1263</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>402</v>
+        <v>1067</v>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="F42" s="8" t="n">
-        <v>6540</v>
+        <v>2275</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>2579792</v>
+        <v>2381480</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>LIBRERIA</t>
+          <t>CONGELADOS HELADOS</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>1822212</v>
+        <v>1770953</v>
       </c>
       <c r="C43" s="8" t="n">
-        <v>748</v>
+        <v>394</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>373</v>
+        <v>348</v>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
@@ -3460,37 +3460,37 @@
         </is>
       </c>
       <c r="F43" s="8" t="n">
-        <v>4885</v>
+        <v>5089</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>1787925</v>
+        <v>1737631</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>HUEVOS FRESCOS</t>
+          <t>LIBRERIA</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>1479800</v>
+        <v>1087282</v>
       </c>
       <c r="C44" s="8" t="n">
-        <v>696</v>
+        <v>403</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>647</v>
+        <v>300</v>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="F44" s="8" t="n">
-        <v>2287</v>
+        <v>3624</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>1451956</v>
+        <v>1066824</v>
       </c>
     </row>
     <row r="45">
@@ -3500,24 +3500,24 @@
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>1375072</v>
+        <v>954045</v>
       </c>
       <c r="C45" s="8" t="n">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>1.1%</t>
         </is>
       </c>
       <c r="F45" s="8" t="n">
-        <v>13481</v>
+        <v>8916</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>1349198</v>
+        <v>936094</v>
       </c>
     </row>
     <row r="46">
@@ -3527,24 +3527,24 @@
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>968460</v>
+        <v>856535</v>
       </c>
       <c r="C46" s="8" t="n">
-        <v>782</v>
+        <v>623</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="F46" s="8" t="n">
-        <v>1784</v>
+        <v>1572</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>950237</v>
+        <v>840418</v>
       </c>
     </row>
     <row r="47">
@@ -3554,267 +3554,267 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>758710</v>
+        <v>823505</v>
       </c>
       <c r="C47" s="8" t="n">
-        <v>430</v>
+        <v>461</v>
       </c>
       <c r="D47" s="8" t="n">
-        <v>305</v>
+        <v>371</v>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>3.1%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="F47" s="8" t="n">
-        <v>2488</v>
+        <v>2220</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>744434</v>
+        <v>808010</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>COTILLON</t>
+          <t>HUEVOS FRESCOS</t>
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>733352</v>
+        <v>809050</v>
       </c>
       <c r="C48" s="8" t="n">
-        <v>332</v>
+        <v>358</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>220</v>
+        <v>358</v>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="F48" s="8" t="n">
-        <v>3333</v>
+        <v>2260</v>
       </c>
       <c r="G48" s="8" t="n">
-        <v>719553</v>
+        <v>793827</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>PESCADOS Y MARISCOS CONGELADOS</t>
+          <t>ENVASES VENTA</t>
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>453910</v>
-      </c>
-      <c r="C49" s="18" t="n">
-        <v>53</v>
-      </c>
-      <c r="D49" s="18" t="n">
-        <v>38</v>
+        <v>659716</v>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>294</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>266</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>0.4%</t>
+          <t>2.8%</t>
         </is>
       </c>
       <c r="F49" s="8" t="n">
-        <v>11945</v>
+        <v>2480</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>445369</v>
+        <v>647303</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>COTILLON</t>
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>435535</v>
+        <v>637188</v>
       </c>
       <c r="C50" s="8" t="n">
-        <v>110</v>
-      </c>
-      <c r="D50" s="18" t="n">
-        <v>86</v>
+        <v>247</v>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>231</v>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>0.9%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="F50" s="8" t="n">
-        <v>5064</v>
+        <v>2758</v>
       </c>
       <c r="G50" s="8" t="n">
-        <v>427340</v>
+        <v>625199</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>CONGELADOS AL 10.5%</t>
+          <t>PESCADOS Y MARISCOS CONGELADOS</t>
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>365292</v>
+        <v>602169</v>
       </c>
       <c r="C51" s="18" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D51" s="18" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>0.5%</t>
+          <t>0.6%</t>
         </is>
       </c>
       <c r="F51" s="8" t="n">
-        <v>8118</v>
+        <v>10206</v>
       </c>
       <c r="G51" s="8" t="n">
-        <v>358419</v>
+        <v>590838</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>FERRETERIA</t>
+          <t>PASCUA</t>
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>328990</v>
-      </c>
-      <c r="C52" s="8" t="n">
-        <v>114</v>
+        <v>462790</v>
+      </c>
+      <c r="C52" s="18" t="n">
+        <v>89</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>0.9%</t>
+          <t>0.7%</t>
         </is>
       </c>
       <c r="F52" s="8" t="n">
-        <v>3655</v>
+        <v>6806</v>
       </c>
       <c r="G52" s="8" t="n">
-        <v>322800</v>
+        <v>454082</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>FACTURAS Y TORTITAS</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="B53" s="8" t="n">
-        <v>244750</v>
-      </c>
-      <c r="C53" s="8" t="n">
-        <v>158</v>
-      </c>
-      <c r="D53" s="8" t="n">
-        <v>137</v>
+        <v>346524</v>
+      </c>
+      <c r="C53" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="D53" s="18" t="n">
+        <v>80</v>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>1.4%</t>
+          <t>0.9%</t>
         </is>
       </c>
       <c r="F53" s="8" t="n">
-        <v>1786</v>
+        <v>4332</v>
       </c>
       <c r="G53" s="8" t="n">
-        <v>240145</v>
+        <v>340004</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>PASCUA</t>
+          <t>CONGELADOS AL 10.5%</t>
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>203670</v>
+        <v>272496</v>
       </c>
       <c r="C54" s="18" t="n">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="D54" s="18" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="F54" s="8" t="n">
-        <v>6570</v>
+        <v>7171</v>
       </c>
       <c r="G54" s="8" t="n">
-        <v>199838</v>
+        <v>267369</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>ZAPATERIA</t>
+          <t>FERRETERIA</t>
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>179900</v>
+        <v>262200</v>
       </c>
       <c r="C55" s="18" t="n">
-        <v>14</v>
+        <v>89</v>
       </c>
       <c r="D55" s="18" t="n">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>0.9%</t>
         </is>
       </c>
       <c r="F55" s="8" t="n">
-        <v>13838</v>
+        <v>3159</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>176515</v>
+        <v>257266</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>PRODUCTOS NAVIDEÑOS</t>
+          <t>ZAPATERIA</t>
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>101950</v>
+        <v>140800</v>
       </c>
       <c r="C56" s="18" t="n">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="D56" s="18" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>0.4%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="F56" s="8" t="n">
-        <v>2913</v>
+        <v>12800</v>
       </c>
       <c r="G56" s="8" t="n">
-        <v>100032</v>
+        <v>138151</v>
       </c>
     </row>
     <row r="57">
@@ -3824,13 +3824,13 @@
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>80148</v>
+        <v>99368</v>
       </c>
       <c r="C57" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D57" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         </is>
       </c>
       <c r="F57" s="8" t="n">
-        <v>11450</v>
+        <v>12421</v>
       </c>
       <c r="G57" s="8" t="n">
-        <v>78639</v>
+        <v>97499</v>
       </c>
     </row>
     <row r="58">
@@ -3851,121 +3851,121 @@
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>63600</v>
+        <v>34900</v>
       </c>
       <c r="C58" s="18" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D58" s="18" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="F58" s="8" t="n">
-        <v>4240</v>
+        <v>4362</v>
       </c>
       <c r="G58" s="8" t="n">
-        <v>62403</v>
+        <v>34243</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>ELECTRODOMESTICOS</t>
+          <t>PRODUCTOS NAVIDEÑOS</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>29850</v>
+        <v>27620</v>
       </c>
       <c r="C59" s="18" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D59" s="18" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="F59" s="8" t="n">
-        <v>14925</v>
+        <v>1534</v>
       </c>
       <c r="G59" s="8" t="n">
-        <v>29288</v>
+        <v>27100</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>MEDICAMENTOS</t>
+          <t>ELECTRODOMESTICOS</t>
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>16560</v>
+        <v>24600</v>
       </c>
       <c r="C60" s="18" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D60" s="18" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="F60" s="8" t="n">
-        <v>1840</v>
+        <v>24600</v>
       </c>
       <c r="G60" s="8" t="n">
-        <v>16248</v>
+        <v>24137</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>ENVASES VENTA</t>
+          <t>IVA RED IB GRAL</t>
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>10533</v>
-      </c>
-      <c r="C61" s="8" t="n">
-        <v>761</v>
-      </c>
-      <c r="D61" s="8" t="n">
-        <v>290</v>
+        <v>16650</v>
+      </c>
+      <c r="C61" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D61" s="18" t="n">
+        <v>9</v>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>2.9%</t>
-        </is>
-      </c>
-      <c r="F61" s="18" t="n">
-        <v>36</v>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="n">
+        <v>1850</v>
       </c>
       <c r="G61" s="8" t="n">
-        <v>10335</v>
+        <v>16337</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>IVA RED IB GRAL</t>
+          <t>HELADOS</t>
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>1850</v>
+        <v>13300</v>
       </c>
       <c r="C62" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D62" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -3973,37 +3973,37 @@
         </is>
       </c>
       <c r="F62" s="8" t="n">
-        <v>1850</v>
+        <v>6650</v>
       </c>
       <c r="G62" s="8" t="n">
-        <v>1815</v>
+        <v>13050</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>PRODUCTOS PARA CARNEO</t>
+          <t>MEDICAMENTOS</t>
         </is>
       </c>
       <c r="B63" s="8" t="n">
-        <v>1650</v>
+        <v>9660</v>
       </c>
       <c r="C63" s="18" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D63" s="18" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="F63" s="8" t="n">
-        <v>1650</v>
+        <v>1380</v>
       </c>
       <c r="G63" s="8" t="n">
-        <v>1619</v>
+        <v>9478</v>
       </c>
     </row>
     <row r="64">
@@ -4013,16 +4013,16 @@
         </is>
       </c>
       <c r="B64" s="12" t="n">
-        <v>355826231</v>
+        <v>318496625</v>
       </c>
       <c r="C64" s="12" t="n">
-        <v>103336</v>
+        <v>82705</v>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
       <c r="E64" s="11" t="inlineStr"/>
       <c r="F64" s="11" t="inlineStr"/>
       <c r="G64" s="12" t="n">
-        <v>349130958</v>
+        <v>312503751</v>
       </c>
     </row>
     <row r="65">
@@ -4084,16 +4084,16 @@
         </is>
       </c>
       <c r="C69" s="8" t="n">
-        <v>11480795</v>
+        <v>10084417</v>
       </c>
       <c r="D69" s="8" t="n">
-        <v>704</v>
+        <v>607</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>841</v>
+        <v>771</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>13651</v>
+        <v>13080</v>
       </c>
       <c r="G69" s="7" t="inlineStr"/>
     </row>
@@ -4109,16 +4109,16 @@
         </is>
       </c>
       <c r="C70" s="8" t="n">
-        <v>8431018</v>
+        <v>8492782</v>
       </c>
       <c r="D70" s="8" t="n">
-        <v>608</v>
+        <v>602</v>
       </c>
       <c r="E70" s="8" t="n">
-        <v>676</v>
+        <v>704</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>12472</v>
+        <v>12064</v>
       </c>
       <c r="G70" s="7" t="inlineStr"/>
     </row>
@@ -4134,141 +4134,141 @@
         </is>
       </c>
       <c r="C71" s="8" t="n">
-        <v>7211831</v>
+        <v>7025746</v>
       </c>
       <c r="D71" s="8" t="n">
-        <v>913</v>
+        <v>889</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>10637</v>
+        <v>10257</v>
       </c>
       <c r="G71" s="7" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>POLLO</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>POLLO AVICOLA LUJAN</t>
+          <t>COSTILLA ARQUEADA</t>
         </is>
       </c>
       <c r="C72" s="8" t="n">
-        <v>6185116</v>
+        <v>5571452</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>1104</v>
+        <v>308</v>
       </c>
       <c r="E72" s="8" t="n">
-        <v>392</v>
+        <v>210</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>15778</v>
+        <v>26531</v>
       </c>
       <c r="G72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>POLLO</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>COSTILLA ARQUEADA</t>
+          <t>POLLO AVICOLA LUJAN</t>
         </is>
       </c>
       <c r="C73" s="8" t="n">
-        <v>5521448</v>
+        <v>5073152</v>
       </c>
       <c r="D73" s="8" t="n">
-        <v>309</v>
+        <v>906</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>204</v>
+        <v>383</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>27066</v>
+        <v>13246</v>
       </c>
       <c r="G73" s="7" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>POLLO</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>FILET / LOMO</t>
+          <t>SUPREMA DE POLLO</t>
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>5167534</v>
+        <v>4792880</v>
       </c>
       <c r="D74" s="8" t="n">
-        <v>208</v>
+        <v>390</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>236</v>
+        <v>421</v>
       </c>
       <c r="F74" s="8" t="n">
-        <v>21896</v>
+        <v>11385</v>
       </c>
       <c r="G74" s="7" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>POLLO</t>
+          <t>ELABORADOS DE CARNICERIA</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>SUPREMA DE POLLO</t>
+          <t>MILANESAS DE POLLO NINO</t>
         </is>
       </c>
       <c r="C75" s="8" t="n">
-        <v>4928426</v>
+        <v>4737150</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>401</v>
+        <v>431</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>11100</v>
+        <v>10411</v>
       </c>
       <c r="G75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>ELABORADOS DE CARNICERIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>MILANESAS DE POLLO NINO</t>
+          <t>FILET / LOMO</t>
         </is>
       </c>
       <c r="C76" s="8" t="n">
-        <v>4864585</v>
+        <v>4197222</v>
       </c>
       <c r="D76" s="8" t="n">
-        <v>442</v>
+        <v>167</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>433</v>
+        <v>206</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>11235</v>
+        <v>20375</v>
       </c>
       <c r="G76" s="7" t="inlineStr"/>
     </row>
@@ -4280,45 +4280,45 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>VACIO</t>
+          <t>NALGA</t>
         </is>
       </c>
       <c r="C77" s="8" t="n">
-        <v>3680860</v>
+        <v>4101204</v>
       </c>
       <c r="D77" s="8" t="n">
-        <v>157</v>
-      </c>
-      <c r="E77" s="18" t="n">
-        <v>93</v>
+        <v>204</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>212</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>39579</v>
+        <v>19345</v>
       </c>
       <c r="G77" s="7" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>ELABORADOS DE CARNICERIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>MILANESAS DE CARNE NINO</t>
+          <t>VACIO</t>
         </is>
       </c>
       <c r="C78" s="8" t="n">
-        <v>3678648</v>
+        <v>3653634</v>
       </c>
       <c r="D78" s="8" t="n">
-        <v>240</v>
-      </c>
-      <c r="E78" s="8" t="n">
-        <v>237</v>
+        <v>155</v>
+      </c>
+      <c r="E78" s="18" t="n">
+        <v>89</v>
       </c>
       <c r="F78" s="8" t="n">
-        <v>15522</v>
+        <v>41052</v>
       </c>
       <c r="G78" s="7" t="inlineStr"/>
     </row>
@@ -4330,45 +4330,45 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>NALGA</t>
+          <t>COSTELETA</t>
         </is>
       </c>
       <c r="C79" s="8" t="n">
-        <v>3676082</v>
+        <v>3483315</v>
       </c>
       <c r="D79" s="8" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>186</v>
+        <v>224</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>19764</v>
+        <v>15551</v>
       </c>
       <c r="G79" s="7" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>ELABORADOS DE CARNICERIA</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>COSTELETA</t>
+          <t>MILANESAS DE CARNE NINO</t>
         </is>
       </c>
       <c r="C80" s="8" t="n">
-        <v>3422754</v>
+        <v>3016338</v>
       </c>
       <c r="D80" s="8" t="n">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="F80" s="8" t="n">
-        <v>14753</v>
+        <v>15234</v>
       </c>
       <c r="G80" s="7" t="inlineStr"/>
     </row>
@@ -4380,20 +4380,20 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>CUADRADA</t>
+          <t>CUADRIL</t>
         </is>
       </c>
       <c r="C81" s="8" t="n">
-        <v>3332272</v>
+        <v>2976877</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>18110</v>
+        <v>18376</v>
       </c>
       <c r="G81" s="7" t="inlineStr"/>
     </row>
@@ -4405,20 +4405,20 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>BOLA LOMO</t>
+          <t>CUADRADA</t>
         </is>
       </c>
       <c r="C82" s="8" t="n">
-        <v>3257059</v>
+        <v>2849548</v>
       </c>
       <c r="D82" s="8" t="n">
-        <v>171</v>
+        <v>148</v>
       </c>
       <c r="E82" s="8" t="n">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="F82" s="8" t="n">
-        <v>17325</v>
+        <v>18384</v>
       </c>
       <c r="G82" s="7" t="inlineStr"/>
     </row>
@@ -4430,20 +4430,20 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>CUADRIL</t>
+          <t>BOLA LOMO</t>
         </is>
       </c>
       <c r="C83" s="8" t="n">
-        <v>3057365</v>
+        <v>2820309</v>
       </c>
       <c r="D83" s="8" t="n">
         <v>146</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>17371</v>
+        <v>17517</v>
       </c>
       <c r="G83" s="7" t="inlineStr"/>
     </row>
@@ -4459,16 +4459,16 @@
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>2541046</v>
+        <v>2400946</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E84" s="18" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F84" s="8" t="n">
-        <v>39093</v>
+        <v>41396</v>
       </c>
       <c r="G84" s="7" t="inlineStr"/>
     </row>
@@ -4480,20 +4480,20 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>PECETO</t>
+          <t>TAPA DE ASADO</t>
         </is>
       </c>
       <c r="C85" s="8" t="n">
-        <v>2366230</v>
+        <v>2384455</v>
       </c>
       <c r="D85" s="8" t="n">
-        <v>112</v>
-      </c>
-      <c r="E85" s="8" t="n">
-        <v>117</v>
+        <v>137</v>
+      </c>
+      <c r="E85" s="18" t="n">
+        <v>91</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>20224</v>
+        <v>26203</v>
       </c>
       <c r="G85" s="7" t="inlineStr"/>
     </row>
@@ -4505,20 +4505,20 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>ASADO CARNICERO-TAPA</t>
+          <t>MAROTILLA</t>
         </is>
       </c>
       <c r="C86" s="8" t="n">
-        <v>2283105</v>
+        <v>2175098</v>
       </c>
       <c r="D86" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="E86" s="18" t="n">
-        <v>72</v>
+        <v>131</v>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>105</v>
       </c>
       <c r="F86" s="8" t="n">
-        <v>31710</v>
+        <v>20715</v>
       </c>
       <c r="G86" s="7" t="inlineStr"/>
     </row>
@@ -4530,245 +4530,245 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>TAPA DE ASADO</t>
+          <t>PECETO</t>
         </is>
       </c>
       <c r="C87" s="8" t="n">
-        <v>2264600</v>
-      </c>
-      <c r="D87" s="8" t="n">
-        <v>132</v>
-      </c>
-      <c r="E87" s="18" t="n">
-        <v>96</v>
+        <v>2071841</v>
+      </c>
+      <c r="D87" s="18" t="n">
+        <v>97</v>
+      </c>
+      <c r="E87" s="8" t="n">
+        <v>103</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>23590</v>
+        <v>20115</v>
       </c>
       <c r="G87" s="7" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>EMBUTIDOS</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>CHORIZO PURO CERDO</t>
+          <t>ASADO CARNICERO-TAPA</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>2244792</v>
-      </c>
-      <c r="D88" s="8" t="n">
-        <v>170</v>
-      </c>
-      <c r="E88" s="8" t="n">
-        <v>298</v>
+        <v>2060964</v>
+      </c>
+      <c r="D88" s="18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E88" s="18" t="n">
+        <v>63</v>
       </c>
       <c r="F88" s="8" t="n">
-        <v>7533</v>
+        <v>32714</v>
       </c>
       <c r="G88" s="7" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>EMBUTIDOS</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>COSTELETA BAJA</t>
+          <t>CHORIZO PURO CERDO</t>
         </is>
       </c>
       <c r="C89" s="8" t="n">
-        <v>2206720</v>
+        <v>2008270</v>
       </c>
       <c r="D89" s="8" t="n">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>165</v>
+        <v>283</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>13374</v>
+        <v>7096</v>
       </c>
       <c r="G89" s="7" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>LACTEOS</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>PALETA</t>
+          <t>SANTA MARIA CREMOSO</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>2143880</v>
+        <v>1997288</v>
       </c>
       <c r="D90" s="8" t="n">
-        <v>113</v>
+        <v>254</v>
       </c>
       <c r="E90" s="8" t="n">
-        <v>124</v>
+        <v>495</v>
       </c>
       <c r="F90" s="8" t="n">
-        <v>17289</v>
+        <v>4035</v>
       </c>
       <c r="G90" s="7" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>ART.DE 1RA NECESIDAD</t>
+          <t>FIAMBRERIA</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>HUEVOS FRESCOS MEDIO MAPLE</t>
+          <t>PALADINI JAMON COCIDO</t>
         </is>
       </c>
       <c r="C91" s="8" t="n">
-        <v>2069900</v>
+        <v>1991669</v>
       </c>
       <c r="D91" s="8" t="n">
-        <v>567</v>
+        <v>116</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>519</v>
+        <v>476</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>3988</v>
+        <v>4184</v>
       </c>
       <c r="G91" s="7" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>FIAMBRERIA</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>PALADINI JAMON COCIDO</t>
+          <t>PALETA</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>2035587</v>
+        <v>1943800</v>
       </c>
       <c r="D92" s="8" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="E92" s="8" t="n">
-        <v>491</v>
+        <v>116</v>
       </c>
       <c r="F92" s="8" t="n">
-        <v>4146</v>
+        <v>16757</v>
       </c>
       <c r="G92" s="7" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>ART.DE 1RA NECESIDAD</t>
+          <t>CARNICERIA AL 10,5 %</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>NATURA ACEITE GRISASOL 1.5 L</t>
+          <t>COSTELETA BAJA</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>1918440</v>
+        <v>1900665</v>
       </c>
       <c r="D93" s="8" t="n">
-        <v>340</v>
+        <v>111</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>324</v>
+        <v>155</v>
       </c>
       <c r="F93" s="8" t="n">
-        <v>5921</v>
+        <v>12262</v>
       </c>
       <c r="G93" s="7" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>ART.DE 1RA NECESIDAD</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>PUNTA DE PIERNA</t>
+          <t>HUEVOS FRESCOS MEDIO MAPLE</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>1896486</v>
-      </c>
-      <c r="D94" s="18" t="n">
-        <v>91</v>
+        <v>1831500</v>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>495</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>109</v>
+        <v>492</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>17399</v>
+        <v>3723</v>
       </c>
       <c r="G94" s="7" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>LACTEOS</t>
+          <t>ART.DE 1RA NECESIDAD</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>SANTA MARIA CREMOSO</t>
+          <t>NATURA ACEITE GRISASOL 1.5 L</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>1893918</v>
+        <v>1797840</v>
       </c>
       <c r="D95" s="8" t="n">
-        <v>245</v>
+        <v>308</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>462</v>
+        <v>308</v>
       </c>
       <c r="F95" s="8" t="n">
-        <v>4099</v>
+        <v>5837</v>
       </c>
       <c r="G95" s="7" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>CARNICERIA AL 10,5 %</t>
+          <t>LACTEOS</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>MAROTILLA</t>
+          <t>BARRA SANTA MARIA</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>1853151</v>
+        <v>1691446</v>
       </c>
       <c r="D96" s="8" t="n">
-        <v>113</v>
-      </c>
-      <c r="E96" s="18" t="n">
-        <v>93</v>
+        <v>150</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>630</v>
       </c>
       <c r="F96" s="8" t="n">
-        <v>19926</v>
+        <v>2685</v>
       </c>
       <c r="G96" s="7" t="inlineStr"/>
     </row>
@@ -4780,20 +4780,20 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>BARRA SANTA MARIA</t>
+          <t>CREMOSO PUNTA DE AGUA</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>1833453</v>
+        <v>1679539</v>
       </c>
       <c r="D97" s="8" t="n">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>655</v>
+        <v>327</v>
       </c>
       <c r="F97" s="8" t="n">
-        <v>2799</v>
+        <v>5136</v>
       </c>
       <c r="G97" s="7" t="inlineStr"/>
     </row>
@@ -4809,16 +4809,16 @@
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>1711927</v>
-      </c>
-      <c r="D98" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="E98" s="8" t="n">
-        <v>107</v>
+        <v>1641906</v>
+      </c>
+      <c r="D98" s="18" t="n">
+        <v>99</v>
+      </c>
+      <c r="E98" s="18" t="n">
+        <v>93</v>
       </c>
       <c r="F98" s="8" t="n">
-        <v>15999</v>
+        <v>17655</v>
       </c>
       <c r="G98" s="7" t="inlineStr"/>
     </row>
@@ -4862,7 +4862,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Periodo: 16/02/2026 - 18/03/2026 (31 dias)</t>
+          <t xml:space="preserve">  Periodo: 01/03/2026 - 31/03/2026 (31 dias)</t>
         </is>
       </c>
     </row>
@@ -4895,10 +4895,10 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>1159</v>
+        <v>1189</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>9983</v>
+        <v>9334</v>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
     </row>
@@ -4909,13 +4909,13 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>11369307</v>
+        <v>10575200</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>28222420</v>
+        <v>20896544</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>39591726</v>
+        <v>31471744</v>
       </c>
     </row>
     <row r="7">
@@ -4925,13 +4925,13 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>54272664</v>
+        <v>51580059</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>355826231</v>
+        <v>318496625</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>410098895</v>
+        <v>370076684</v>
       </c>
     </row>
     <row r="8">
@@ -4941,13 +4941,13 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>65641971</v>
+        <v>62155259</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>384048650</v>
+        <v>339393168</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>449690621</v>
+        <v>401548427</v>
       </c>
     </row>
     <row r="9">
@@ -4958,12 +4958,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>4.8x</t>
+          <t>4.9x</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>12.6x</t>
+          <t>15.2x</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr"/>
@@ -4975,10 +4975,10 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>56637</v>
+        <v>52275</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>38470</v>
+        <v>36361</v>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
     </row>
@@ -4989,10 +4989,10 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>31175</v>
+        <v>28718</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>28286</v>
+        <v>25978</v>
       </c>
       <c r="D11" s="7" t="inlineStr"/>
     </row>
@@ -5032,13 +5032,13 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>11155381</v>
+        <v>10376216</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>27691383</v>
+        <v>20503352</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>38846764</v>
+        <v>30879568</v>
       </c>
     </row>
     <row r="16">
@@ -5048,13 +5048,13 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>53251462</v>
+        <v>50609522</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>349130958</v>
+        <v>312503751</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>402382420</v>
+        <v>363113273</v>
       </c>
     </row>
     <row r="17">
@@ -5064,13 +5064,13 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>64406843</v>
+        <v>60985738</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>376822341</v>
+        <v>333007103</v>
       </c>
       <c r="D17" s="12" t="n">
-        <v>441229184</v>
+        <v>393992841</v>
       </c>
     </row>
     <row r="19">

</xml_diff>